<commit_message>
Added or updated results
</commit_message>
<xml_diff>
--- a/results-summarized/summary-German-morf-xsk.xlsx
+++ b/results-summarized/summary-German-morf-xsk.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kowk/Dropbox/GitHub/ngram-based-noun-classification/results/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kowk/Dropbox/GitHub/ngram-based-noun-classification/results-summarized/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C10F5908-F707-D74D-B0CA-B3A382CB8424}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D97F470A-2432-A04F-A15C-B6D59FD7AF8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4520" yWindow="1880" windowWidth="30360" windowHeight="17420" xr2:uid="{F93E9898-A028-3840-BE37-DF8ADAD35830}"/>
+    <workbookView xWindow="5980" yWindow="3020" windowWidth="30360" windowHeight="17420" xr2:uid="{F93E9898-A028-3840-BE37-DF8ADAD35830}"/>
   </bookViews>
   <sheets>
     <sheet name="summarized" sheetId="7" r:id="rId1"/>

</xml_diff>